<commit_message>
docs(testing): address seeded case review findings
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 211026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 211026.xlsx
@@ -2291,17 +2291,17 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Seeded "Jasmine Hall" has a Confirmed booking for coord_a's "EVT-3001 Approved Annual Conference" on 15/10/2026; coord_b@connectsphere.com is signed in and is not assigned to the event</t>
+          <t>The seed has EVT-3003, owned by coord_a@connectsphere.com, with a Pending Orchid Hall booking on 25/10/2026. For this case only, prepare the event and booking as Confirmed while retaining coord_a ownership; coord_b@connectsphere.com is signed in and is not assigned to the event.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>1. Open the availability calendar for "Jasmine Hall" on 15/10/2026</t>
+          <t>1. Open the availability calendar for Orchid Hall on 25/10/2026</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Seeded booking for another Coordinator: EVT-3001 at Jasmine Hall on 15/10/2026</t>
+          <t>Future seeded booking for another Coordinator, prepared for this case: EVT-3003 at Orchid Hall on 25/10/2026, Confirmed and still assigned to coord_a@connectsphere.com</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -18589,13 +18589,13 @@
       </c>
       <c r="H347" s="2" t="inlineStr">
         <is>
-          <t>1. As coord_a@connectsphere.com, edit the effective event date or time while keeping the venue at Jasmine Hall
+          <t>1. As coord_a@connectsphere.com, change the effective event date/time to a future date and time while keeping the venue at Jasmine Hall
   2. Check notifications for organiser_a@clienta.com, venue_b@connectsphere.com, tech_a@connectsphere.com, attendee_a@example.com, and attendee_b@example.com</t>
         </is>
       </c>
       <c r="I347" s="2" t="inlineStr">
         <is>
-          <t>Changed field: Effective date/time; venue unchanged (Jasmine Hall)</t>
+          <t>Changed field: Effective date/time (set to a future period, e.g. 26/10/2026, 09:00–17:00); venue unchanged (Jasmine Hall)</t>
         </is>
       </c>
       <c r="J347" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(testing): align E11 notification fixtures (SCRUM-179)
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 211026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 211026.xlsx
@@ -18533,23 +18533,23 @@
       </c>
       <c r="G346" s="2" t="inlineStr">
         <is>
-          <t>organiser_a@clienta.com is linked to event "EVT-3001 Approved Annual Conference", currently "Under Review"</t>
+          <t>organiser_c@clientb.com is linked to seeded event "EVT-2003 Client B Isolation Event", currently "Under Review"; coord_b@connectsphere.com is its assigned Coordinator</t>
         </is>
       </c>
       <c r="H346" s="2" t="inlineStr">
         <is>
-          <t>1. As coord_a@connectsphere.com, approve request "EVT-3001 Approved Annual Conference" (status -&gt; Approved)
-  2. Log in as organiser_a@clienta.com and open notifications</t>
+          <t>1. As coord_b@connectsphere.com, approve request "EVT-2003 Client B Isolation Event" (status -&gt; Approved)
+  2. Log in as organiser_c@clientb.com and open notifications</t>
         </is>
       </c>
       <c r="I346" s="2" t="inlineStr">
         <is>
-          <t>Event: Annual Tech Summit | Change: Under Review -&gt; Approved</t>
+          <t>Event: EVT-2003 Client B Isolation Event | Change: Under Review -&gt; Approved</t>
         </is>
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>A notification is received stating the status changed to "Approved", the time of the change, and that it concerns "EVT-3001 Approved Annual Conference"</t>
+          <t>A notification is received stating the status changed to "Approved", the time of the change, and that it concerns "EVT-2003 Client B Isolation Event"</t>
         </is>
       </c>
     </row>

</xml_diff>